<commit_message>
paper run 2026-09-11 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-11.xlsx
+++ b/reports/2026-09-11.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,6 +601,178 @@
       </c>
       <c r="K4" t="n">
         <v>4.7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-11T14:26:22.427541+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F5" t="n">
+        <v>32.45</v>
+      </c>
+      <c r="G5" t="n">
+        <v>55</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00198</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>22.55</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-11T15:41:50.726445+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00127</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-11T16:34:04.466449+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F7" t="n">
+        <v>42.18</v>
+      </c>
+      <c r="G7" t="n">
+        <v>82.70999999999999</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00128</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>40.53</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-11T16:41:21.298590+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F8" t="n">
+        <v>44.21</v>
+      </c>
+      <c r="G8" t="n">
+        <v>86.68000000000001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00118</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>42.47</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,7 +808,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -646,7 +818,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -656,7 +828,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -666,7 +838,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="6">
@@ -676,7 +848,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-29.02</v>
+        <v>73.53</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14.1</v>
+        <v>119.65</v>
       </c>
     </row>
     <row r="8">
@@ -696,7 +868,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-43.12</v>
+        <v>-46.12</v>
       </c>
     </row>
     <row r="9">
@@ -706,7 +878,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.33</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +888,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>824.0700000000001</v>
+        <v>926.62</v>
       </c>
     </row>
     <row r="12">
@@ -767,16 +939,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>-7.04</v>
+        <v>172.24</v>
       </c>
       <c r="E15" t="n">
-        <v>-38.42</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="16">
@@ -786,16 +958,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D16" t="n">
-        <v>37.83</v>
+        <v>186.08</v>
       </c>
       <c r="E16" t="n">
-        <v>9.4</v>
+        <v>49.93</v>
       </c>
     </row>
     <row r="17">
@@ -812,13 +984,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>-7.04</v>
+        <v>65.27</v>
       </c>
       <c r="E18" t="n">
         <v>-38.42</v>
@@ -827,358 +999,393 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>37.83</v>
+        <v>73.01000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>9.4</v>
+        <v>62.02</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>120.83</v>
+      </c>
+      <c r="E20" t="n">
+        <v>49.93</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>73.91</v>
+        <v>99.20999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>14.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-43.12</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-43.12</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9</v>
+      </c>
+      <c r="C23" t="n">
+        <v>9</v>
+      </c>
+      <c r="D23" t="n">
+        <v>353.48</v>
+      </c>
+      <c r="E23" t="n">
+        <v>97.09999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>81.05</v>
+      </c>
+      <c r="E24" t="n">
+        <v>19.55</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
         <v>2</v>
       </c>
-      <c r="D24" t="n">
-        <v>30.79</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-29.02</v>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-76.20999999999999</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-43.12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>125.47</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" t="n">
+        <v>129.05</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D29" t="n">
-        <v>-38.42</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+        <v>103.8</v>
+      </c>
+      <c r="E29" t="n">
+        <v>73.53</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>-38.42</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>9.4</v>
+        <v>-38.42</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="n">
+        <v>62.02</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>9.4</v>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>49.93</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-38.42</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>23.6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
         <v>2</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C40" t="n">
         <v>2</v>
       </c>
-      <c r="D41" t="n">
-        <v>14.1</v>
+      <c r="D40" t="n">
+        <v>49.93</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
         <v>1</v>
       </c>
-      <c r="C42" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" t="n">
-        <v>-43.12</v>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-38.42</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>14.1</v>
+        <v>22.55</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1188,61 +1395,217 @@
         <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>-43.12</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>2</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>-33.72</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>97.09999999999999</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>19.55</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-43.12</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" t="n">
+        <v>56.57</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-5.59</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>22.55</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>-33.72</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>4.7</v>
+      <c r="B61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>107.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-11 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-11.xlsx
+++ b/reports/2026-09-11.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -773,6 +773,92 @@
       </c>
       <c r="K8" t="n">
         <v>42.47</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-11T22:11:15.974678+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F9" t="n">
+        <v>21.35</v>
+      </c>
+      <c r="G9" t="n">
+        <v>35</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.00149</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>13.65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-11T23:11:46.243570+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F10" t="n">
+        <v>45.34</v>
+      </c>
+      <c r="G10" t="n">
+        <v>88.91</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.00103</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>43.57</v>
       </c>
     </row>
   </sheetData>
@@ -786,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,7 +894,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -818,7 +904,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -838,7 +924,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="6">
@@ -848,7 +934,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>73.53</v>
+        <v>130.75</v>
       </c>
     </row>
     <row r="7">
@@ -858,7 +944,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>119.65</v>
+        <v>176.87</v>
       </c>
     </row>
     <row r="8">
@@ -878,7 +964,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.59</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="10">
@@ -888,7 +974,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>926.62</v>
+        <v>983.8399999999999</v>
       </c>
     </row>
     <row r="12">
@@ -939,16 +1025,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D15" t="n">
-        <v>172.24</v>
+        <v>331.16</v>
       </c>
       <c r="E15" t="n">
-        <v>23.6</v>
+        <v>80.81999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -958,13 +1044,13 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="n">
         <v>7</v>
       </c>
-      <c r="C16" t="n">
-        <v>6</v>
-      </c>
       <c r="D16" t="n">
-        <v>186.08</v>
+        <v>220.13</v>
       </c>
       <c r="E16" t="n">
         <v>49.93</v>
@@ -984,16 +1070,16 @@
         </is>
       </c>
       <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
         <v>4</v>
       </c>
-      <c r="C18" t="n">
-        <v>3</v>
-      </c>
       <c r="D18" t="n">
-        <v>65.27</v>
+        <v>110.44</v>
       </c>
       <c r="E18" t="n">
-        <v>-38.42</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="19">
@@ -1003,16 +1089,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>73.01000000000001</v>
+        <v>134.58</v>
       </c>
       <c r="E19" t="n">
-        <v>62.02</v>
+        <v>75.67</v>
       </c>
     </row>
     <row r="20">
@@ -1022,13 +1108,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>120.83</v>
+        <v>184.87</v>
       </c>
       <c r="E20" t="n">
         <v>49.93</v>
@@ -1041,13 +1127,13 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
       <c r="D21" t="n">
-        <v>99.20999999999999</v>
+        <v>121.4</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -1067,16 +1153,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>353.48</v>
+        <v>398.65</v>
       </c>
       <c r="E23" t="n">
-        <v>97.09999999999999</v>
+        <v>140.67</v>
       </c>
     </row>
     <row r="24">
@@ -1086,13 +1172,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>81.05</v>
+        <v>181.49</v>
       </c>
       <c r="E24" t="n">
         <v>19.55</v>
@@ -1105,16 +1191,16 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
         <v>2</v>
       </c>
-      <c r="C25" t="n">
-        <v>0</v>
-      </c>
       <c r="D25" t="n">
-        <v>-76.20999999999999</v>
+        <v>-28.85</v>
       </c>
       <c r="E25" t="n">
-        <v>-43.12</v>
+        <v>-29.47</v>
       </c>
     </row>
     <row r="26">
@@ -1150,13 +1236,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>129.05</v>
+        <v>251.68</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1169,16 +1255,16 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C29" t="n">
         <v>7</v>
       </c>
-      <c r="C29" t="n">
-        <v>5</v>
-      </c>
       <c r="D29" t="n">
-        <v>103.8</v>
+        <v>174.14</v>
       </c>
       <c r="E29" t="n">
-        <v>73.53</v>
+        <v>130.75</v>
       </c>
     </row>
     <row r="31">
@@ -1217,13 +1303,13 @@
         </is>
       </c>
       <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="n">
         <v>2</v>
       </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
       <c r="D34" t="n">
-        <v>-38.42</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="35">
@@ -1233,13 +1319,13 @@
         </is>
       </c>
       <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
         <v>3</v>
       </c>
-      <c r="C35" t="n">
-        <v>2</v>
-      </c>
       <c r="D35" t="n">
-        <v>62.02</v>
+        <v>75.67</v>
       </c>
     </row>
     <row r="36">
@@ -1287,13 +1373,13 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="C39" t="n">
-        <v>3</v>
-      </c>
       <c r="D39" t="n">
-        <v>23.6</v>
+        <v>80.81999999999999</v>
       </c>
     </row>
     <row r="40">
@@ -1414,198 +1500,230 @@
         <v>83</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>13.65</v>
+      </c>
+    </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>4</v>
-      </c>
-      <c r="C50" t="n">
-        <v>4</v>
-      </c>
-      <c r="D50" t="n">
-        <v>97.09999999999999</v>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>43.57</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="n">
-        <v>19.55</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B52" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" t="n">
+        <v>5</v>
+      </c>
+      <c r="D52" t="n">
+        <v>140.67</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
         <v>1</v>
       </c>
-      <c r="C52" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" t="n">
-        <v>-43.12</v>
+      <c r="D53" t="n">
+        <v>19.55</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>3</v>
-      </c>
-      <c r="C55" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" t="n">
-        <v>56.57</v>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>-29.47</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="n">
-        <v>-5.59</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D57" t="n">
-        <v>22.55</v>
+        <v>100.14</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>8.06</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>2</v>
-      </c>
-      <c r="C60" t="n">
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
         <v>1</v>
       </c>
-      <c r="D60" t="n">
-        <v>-33.72</v>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>22.55</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="n">
+        <v>-33.72</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B61" t="n">
-        <v>5</v>
-      </c>
-      <c r="C61" t="n">
-        <v>4</v>
-      </c>
-      <c r="D61" t="n">
-        <v>107.25</v>
+      <c r="B63" t="n">
+        <v>7</v>
+      </c>
+      <c r="C63" t="n">
+        <v>6</v>
+      </c>
+      <c r="D63" t="n">
+        <v>164.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>